<commit_message>
LithoLog milestone 3: contour maps, 3D block model, volumes and storage
- grid: per-borehole attributes (ground, top/base/depth/thickness of a
  unit, water table, depth to water); IDW, linear and ordinary kriging
  (fitted spherical variogram); convex-hull masking; ESRI ASCII export
- maps: contour maps with labelled boreholes, flow arrows on water-table
  maps, isopach volume, colour bar, north arrow, scale bar
- model3d: indicator-IDW voxel model (depth or elevation datum), volumes
  from vote proportions so thin units are not under-counted, storage
  from user specific yield, cut-away and per-unit 3D views, horizontal
  slices, VTK export
- CLI 'map' and 'model' commands; tests; README; demo boreholes spread
  out so the demo maps are meaningful

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M7uSz71TnHaAoXYBsjNkTJ
</commit_message>
<xml_diff>
--- a/litholog/examples/sample_project.xlsx
+++ b/litholog/examples/sample_project.xlsx
@@ -540,10 +540,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>651640</v>
+        <v>652150</v>
       </c>
       <c r="C3" t="n">
-        <v>1688120</v>
+        <v>1688600</v>
       </c>
       <c r="D3" t="n">
         <v>481.7</v>
@@ -577,10 +577,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>652010</v>
+        <v>651700</v>
       </c>
       <c r="C4" t="n">
-        <v>1687760</v>
+        <v>1687800</v>
       </c>
       <c r="D4" t="n">
         <v>476.9</v>
@@ -614,10 +614,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>652480</v>
+        <v>652650</v>
       </c>
       <c r="C5" t="n">
-        <v>1687430</v>
+        <v>1687550</v>
       </c>
       <c r="D5" t="n">
         <v>472.3</v>
@@ -651,10 +651,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>652900</v>
+        <v>651250</v>
       </c>
       <c r="C6" t="n">
-        <v>1687010</v>
+        <v>1687050</v>
       </c>
       <c r="D6" t="n">
         <v>468.8</v>
@@ -688,10 +688,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>653420</v>
+        <v>652450</v>
       </c>
       <c r="C7" t="n">
-        <v>1686540</v>
+        <v>1686750</v>
       </c>
       <c r="D7" t="n">
         <v>459.4</v>

</xml_diff>

<commit_message>
LithoLog: aquifer, property, stratigraphy, hydrochemistry, log-section and fracture engines
- aquifer: observation wells (long/wide/seasonal tables, X/Y or lat/lon
  with conversion), water table on the model grid, saturated volumes and
  storage per unit, saturated thickness
- property3d: anisotropic 3D IDW of downhole values (log space for
  resistivity-like data), slices, volume-in-range, Plotly volume, VTK
- strat: ordered formation tops -> non-crossing surfaces -> block model
- hydrochem: ionic balance, water type, SAR/%Na/RSC/Kelly/PI/MH; Piper,
  Durov, Stiff, USSL (Richards 1954), Wilcox (1955) classes, Gibbs
- sections: log-section style with depth ticks and downhole curve tracks
- fractures: Fractures sheet; rose, equal-area stereonet with density,
  frequency with water strikes; tadpole track on strip logs
- demo data gains fractures

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M7uSz71TnHaAoXYBsjNkTJ
</commit_message>
<xml_diff>
--- a/litholog/examples/sample_project.xlsx
+++ b/litholog/examples/sample_project.xlsx
@@ -13,6 +13,7 @@
     <sheet name="Construction" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="WaterLevels" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Downhole" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Fractures" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -11599,4 +11600,1340 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G52"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Borehole ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Depth (m)</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Dip (deg)</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Dip direction (deg)</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Aperture (mm)</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Yield (lps)</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>BW-01</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="C2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D2" t="n">
+        <v>243</v>
+      </c>
+      <c r="E2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>BW-01</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="C3" t="n">
+        <v>15</v>
+      </c>
+      <c r="D3" t="n">
+        <v>278</v>
+      </c>
+      <c r="E3" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>BW-01</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="C4" t="n">
+        <v>61</v>
+      </c>
+      <c r="D4" t="n">
+        <v>136</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>BW-01</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="C5" t="n">
+        <v>64</v>
+      </c>
+      <c r="D5" t="n">
+        <v>125</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>BW-01</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="C6" t="n">
+        <v>11</v>
+      </c>
+      <c r="D6" t="n">
+        <v>209</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>BW-01</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="C7" t="n">
+        <v>72</v>
+      </c>
+      <c r="D7" t="n">
+        <v>137</v>
+      </c>
+      <c r="E7" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>BW-01</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>15.3</v>
+      </c>
+      <c r="C8" t="n">
+        <v>16</v>
+      </c>
+      <c r="D8" t="n">
+        <v>202</v>
+      </c>
+      <c r="E8" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="F8" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Water strike</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>BW-01</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="C9" t="n">
+        <v>79</v>
+      </c>
+      <c r="D9" t="n">
+        <v>143</v>
+      </c>
+      <c r="E9" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>BW-01</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="C10" t="n">
+        <v>8</v>
+      </c>
+      <c r="D10" t="n">
+        <v>225</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>BW-01</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>52.3</v>
+      </c>
+      <c r="C11" t="n">
+        <v>63</v>
+      </c>
+      <c r="D11" t="n">
+        <v>134</v>
+      </c>
+      <c r="E11" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>BW-01</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>54.7</v>
+      </c>
+      <c r="C12" t="n">
+        <v>5</v>
+      </c>
+      <c r="D12" t="n">
+        <v>244</v>
+      </c>
+      <c r="E12" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>BW-02</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="C13" t="n">
+        <v>76</v>
+      </c>
+      <c r="D13" t="n">
+        <v>133</v>
+      </c>
+      <c r="E13" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>BW-02</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="C14" t="n">
+        <v>4</v>
+      </c>
+      <c r="D14" t="n">
+        <v>142</v>
+      </c>
+      <c r="E14" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>BW-02</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="C15" t="n">
+        <v>74</v>
+      </c>
+      <c r="D15" t="n">
+        <v>147</v>
+      </c>
+      <c r="E15" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>BW-02</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="C16" t="n">
+        <v>73</v>
+      </c>
+      <c r="D16" t="n">
+        <v>140</v>
+      </c>
+      <c r="E16" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>BW-02</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="C17" t="n">
+        <v>13</v>
+      </c>
+      <c r="D17" t="n">
+        <v>151</v>
+      </c>
+      <c r="E17" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>BW-02</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="C18" t="n">
+        <v>76</v>
+      </c>
+      <c r="D18" t="n">
+        <v>112</v>
+      </c>
+      <c r="E18" t="n">
+        <v>2</v>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>BW-02</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>13.1</v>
+      </c>
+      <c r="C19" t="n">
+        <v>20</v>
+      </c>
+      <c r="D19" t="n">
+        <v>185</v>
+      </c>
+      <c r="E19" t="n">
+        <v>4</v>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>BW-02</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="C20" t="n">
+        <v>89</v>
+      </c>
+      <c r="D20" t="n">
+        <v>133</v>
+      </c>
+      <c r="E20" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>BW-02</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>15.3</v>
+      </c>
+      <c r="C21" t="n">
+        <v>73</v>
+      </c>
+      <c r="D21" t="n">
+        <v>115</v>
+      </c>
+      <c r="E21" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>BW-02</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>17.1</v>
+      </c>
+      <c r="C22" t="n">
+        <v>81</v>
+      </c>
+      <c r="D22" t="n">
+        <v>139</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>BW-02</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="C23" t="n">
+        <v>72</v>
+      </c>
+      <c r="D23" t="n">
+        <v>129</v>
+      </c>
+      <c r="E23" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Water strike</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>BW-02</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>20.7</v>
+      </c>
+      <c r="C24" t="n">
+        <v>72</v>
+      </c>
+      <c r="D24" t="n">
+        <v>146</v>
+      </c>
+      <c r="E24" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>BW-03</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="C25" t="n">
+        <v>6</v>
+      </c>
+      <c r="D25" t="n">
+        <v>234</v>
+      </c>
+      <c r="E25" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>BW-03</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>20.2</v>
+      </c>
+      <c r="C26" t="n">
+        <v>14</v>
+      </c>
+      <c r="D26" t="n">
+        <v>191</v>
+      </c>
+      <c r="E26" t="n">
+        <v>3</v>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>BW-03</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>22</v>
+      </c>
+      <c r="C27" t="n">
+        <v>77</v>
+      </c>
+      <c r="D27" t="n">
+        <v>134</v>
+      </c>
+      <c r="E27" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>BW-03</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="C28" t="n">
+        <v>80</v>
+      </c>
+      <c r="D28" t="n">
+        <v>124</v>
+      </c>
+      <c r="E28" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>BW-03</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="C29" t="n">
+        <v>6</v>
+      </c>
+      <c r="D29" t="n">
+        <v>128</v>
+      </c>
+      <c r="E29" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="F29" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Water strike</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>BW-03</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>64.3</v>
+      </c>
+      <c r="C30" t="n">
+        <v>63</v>
+      </c>
+      <c r="D30" t="n">
+        <v>126</v>
+      </c>
+      <c r="E30" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>BW-03</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>67.7</v>
+      </c>
+      <c r="C31" t="n">
+        <v>66</v>
+      </c>
+      <c r="D31" t="n">
+        <v>142</v>
+      </c>
+      <c r="E31" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>BW-04</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="C32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D32" t="n">
+        <v>152</v>
+      </c>
+      <c r="E32" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>BW-04</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="C33" t="n">
+        <v>69</v>
+      </c>
+      <c r="D33" t="n">
+        <v>138</v>
+      </c>
+      <c r="E33" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>BW-04</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="C34" t="n">
+        <v>72</v>
+      </c>
+      <c r="D34" t="n">
+        <v>158</v>
+      </c>
+      <c r="E34" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>BW-04</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="C35" t="n">
+        <v>64</v>
+      </c>
+      <c r="D35" t="n">
+        <v>119</v>
+      </c>
+      <c r="E35" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>BW-04</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="C36" t="n">
+        <v>6</v>
+      </c>
+      <c r="D36" t="n">
+        <v>144</v>
+      </c>
+      <c r="E36" t="n">
+        <v>4</v>
+      </c>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>BW-04</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="C37" t="n">
+        <v>49</v>
+      </c>
+      <c r="D37" t="n">
+        <v>141</v>
+      </c>
+      <c r="E37" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>BW-04</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="C38" t="n">
+        <v>63</v>
+      </c>
+      <c r="D38" t="n">
+        <v>132</v>
+      </c>
+      <c r="E38" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="F38" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Water strike</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>BW-04</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="C39" t="n">
+        <v>69</v>
+      </c>
+      <c r="D39" t="n">
+        <v>125</v>
+      </c>
+      <c r="E39" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="F39" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Water strike</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>BW-04</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="C40" t="n">
+        <v>11</v>
+      </c>
+      <c r="D40" t="n">
+        <v>155</v>
+      </c>
+      <c r="E40" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>BW-04</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>31.3</v>
+      </c>
+      <c r="C41" t="n">
+        <v>87</v>
+      </c>
+      <c r="D41" t="n">
+        <v>133</v>
+      </c>
+      <c r="E41" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>BW-04</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>33.4</v>
+      </c>
+      <c r="C42" t="n">
+        <v>67</v>
+      </c>
+      <c r="D42" t="n">
+        <v>126</v>
+      </c>
+      <c r="E42" t="n">
+        <v>4</v>
+      </c>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>BW-04</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>35.6</v>
+      </c>
+      <c r="C43" t="n">
+        <v>16</v>
+      </c>
+      <c r="D43" t="n">
+        <v>196</v>
+      </c>
+      <c r="E43" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>BW-04</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>37.7</v>
+      </c>
+      <c r="C44" t="n">
+        <v>8</v>
+      </c>
+      <c r="D44" t="n">
+        <v>162</v>
+      </c>
+      <c r="E44" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>BW-05</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>58.3</v>
+      </c>
+      <c r="C45" t="n">
+        <v>13</v>
+      </c>
+      <c r="D45" t="n">
+        <v>200</v>
+      </c>
+      <c r="E45" t="n">
+        <v>2</v>
+      </c>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>BW-05</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>59.9</v>
+      </c>
+      <c r="C46" t="n">
+        <v>61</v>
+      </c>
+      <c r="D46" t="n">
+        <v>128</v>
+      </c>
+      <c r="E46" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>BW-05</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>61.6</v>
+      </c>
+      <c r="C47" t="n">
+        <v>73</v>
+      </c>
+      <c r="D47" t="n">
+        <v>137</v>
+      </c>
+      <c r="E47" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>BW-05</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>63.2</v>
+      </c>
+      <c r="C48" t="n">
+        <v>69</v>
+      </c>
+      <c r="D48" t="n">
+        <v>123</v>
+      </c>
+      <c r="E48" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>BW-05</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>64.8</v>
+      </c>
+      <c r="C49" t="n">
+        <v>73</v>
+      </c>
+      <c r="D49" t="n">
+        <v>121</v>
+      </c>
+      <c r="E49" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>BW-05</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>66.40000000000001</v>
+      </c>
+      <c r="C50" t="n">
+        <v>75</v>
+      </c>
+      <c r="D50" t="n">
+        <v>133</v>
+      </c>
+      <c r="E50" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>BW-05</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>68.09999999999999</v>
+      </c>
+      <c r="C51" t="n">
+        <v>59</v>
+      </c>
+      <c r="D51" t="n">
+        <v>141</v>
+      </c>
+      <c r="E51" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>BW-05</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>69.7</v>
+      </c>
+      <c r="C52" t="n">
+        <v>14</v>
+      </c>
+      <c r="D52" t="n">
+        <v>174</v>
+      </c>
+      <c r="E52" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>